<commit_message>
PIX: data do PDV é dia de movimento; caça cartão lançado como PIX (caso ROBS 12/10 R$ 59,50)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XeuzNyreGoe8Jd1wBUgeX
</commit_message>
<xml_diff>
--- a/saida/concilia_pix_2026-10-08_a_2026-10-14.xlsx
+++ b/saida/concilia_pix_2026-10-08_a_2026-10-14.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="185">
   <si>
     <t>Filial</t>
   </si>
@@ -59,6 +59,9 @@
     <t>92357491</t>
   </si>
   <si>
+    <t>Dia movimento</t>
+  </si>
+  <si>
     <t>Hora</t>
   </si>
   <si>
@@ -275,7 +278,7 @@
     <t>CONCILIADO</t>
   </si>
   <si>
-    <t>SEM PAR NA MAQUININHA</t>
+    <t>PROVÁVEL FORMA ERRADA: Crédito Mastercard na máquina em 11/10 22:33</t>
   </si>
   <si>
     <t>20:38:48</t>
@@ -353,6 +356,9 @@
     <t>23:05:22</t>
   </si>
   <si>
+    <t>22:33:58</t>
+  </si>
+  <si>
     <t>21:27:50</t>
   </si>
   <si>
@@ -437,6 +443,9 @@
     <t>SE000000589830GDV6WMCR7ZQ0095IB3YK</t>
   </si>
   <si>
+    <t>340070</t>
+  </si>
+  <si>
     <t>SE0010000000004SEAFME2OR685COMIXY0</t>
   </si>
   <si>
@@ -534,6 +543,9 @@
   </si>
   <si>
     <t>000003</t>
+  </si>
+  <si>
+    <t>000001626</t>
   </si>
   <si>
     <t>006806</t>
@@ -1186,10 +1198,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1232,8 +1244,11 @@
       <c r="N1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1243,41 +1258,44 @@
       <c r="C2" s="1">
         <v>46303</v>
       </c>
-      <c r="D2" t="s">
-        <v>24</v>
+      <c r="D2" s="1">
+        <v>46303</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="G2" t="s">
         <v>83</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2">
         <v>34.4</v>
       </c>
-      <c r="I2" t="s">
-        <v>84</v>
-      </c>
       <c r="J2" t="s">
-        <v>86</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2" t="s">
-        <v>114</v>
+        <v>85</v>
+      </c>
+      <c r="K2" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>142</v>
+        <v>116</v>
       </c>
       <c r="N2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1287,41 +1305,44 @@
       <c r="C3" s="1">
         <v>46303</v>
       </c>
-      <c r="D3" t="s">
-        <v>25</v>
+      <c r="D3" s="1">
+        <v>46303</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="G3" t="s">
         <v>83</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I3">
         <v>49.2</v>
       </c>
-      <c r="I3" t="s">
-        <v>84</v>
-      </c>
       <c r="J3" t="s">
-        <v>87</v>
-      </c>
-      <c r="K3">
+        <v>85</v>
+      </c>
+      <c r="K3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L3">
         <v>10</v>
       </c>
-      <c r="L3" t="s">
-        <v>115</v>
-      </c>
       <c r="M3" t="s">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="N3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1331,41 +1352,44 @@
       <c r="C4" s="1">
         <v>46303</v>
       </c>
-      <c r="D4" t="s">
-        <v>26</v>
+      <c r="D4" s="1">
+        <v>46303</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
         <v>83</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4">
         <v>10.95</v>
       </c>
-      <c r="I4" t="s">
-        <v>84</v>
-      </c>
       <c r="J4" t="s">
-        <v>88</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4" t="s">
-        <v>116</v>
+        <v>85</v>
+      </c>
+      <c r="K4" t="s">
+        <v>89</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
       </c>
       <c r="M4" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="N4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1375,41 +1399,44 @@
       <c r="C5" s="1">
         <v>46304</v>
       </c>
-      <c r="D5" t="s">
-        <v>27</v>
+      <c r="D5" s="1">
+        <v>46304</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="G5" t="s">
         <v>83</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I5">
         <v>115.65</v>
       </c>
-      <c r="I5" t="s">
-        <v>84</v>
-      </c>
       <c r="J5" t="s">
-        <v>89</v>
-      </c>
-      <c r="K5">
+        <v>85</v>
+      </c>
+      <c r="K5" t="s">
+        <v>90</v>
+      </c>
+      <c r="L5">
         <v>1</v>
       </c>
-      <c r="L5" t="s">
-        <v>117</v>
-      </c>
       <c r="M5" t="s">
-        <v>142</v>
+        <v>119</v>
       </c>
       <c r="N5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1419,41 +1446,44 @@
       <c r="C6" s="1">
         <v>46304</v>
       </c>
-      <c r="D6" t="s">
-        <v>28</v>
+      <c r="D6" s="1">
+        <v>46304</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="G6" t="s">
         <v>83</v>
       </c>
-      <c r="H6">
+      <c r="H6" t="s">
+        <v>84</v>
+      </c>
+      <c r="I6">
         <v>33.25</v>
       </c>
-      <c r="I6" t="s">
-        <v>84</v>
-      </c>
       <c r="J6" t="s">
-        <v>90</v>
-      </c>
-      <c r="K6">
+        <v>85</v>
+      </c>
+      <c r="K6" t="s">
+        <v>91</v>
+      </c>
+      <c r="L6">
         <v>45</v>
       </c>
-      <c r="L6" t="s">
-        <v>118</v>
-      </c>
       <c r="M6" t="s">
-        <v>144</v>
+        <v>120</v>
       </c>
       <c r="N6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>147</v>
+      </c>
+      <c r="O6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1463,41 +1493,44 @@
       <c r="C7" s="1">
         <v>46304</v>
       </c>
-      <c r="D7" t="s">
-        <v>29</v>
+      <c r="D7" s="1">
+        <v>46304</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="G7" t="s">
         <v>83</v>
       </c>
-      <c r="H7">
+      <c r="H7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I7">
         <v>34.45</v>
       </c>
-      <c r="I7" t="s">
-        <v>84</v>
-      </c>
       <c r="J7" t="s">
-        <v>91</v>
-      </c>
-      <c r="K7">
+        <v>85</v>
+      </c>
+      <c r="K7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L7">
         <v>10</v>
       </c>
-      <c r="L7" t="s">
-        <v>119</v>
-      </c>
       <c r="M7" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="N7" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1507,41 +1540,44 @@
       <c r="C8" s="1">
         <v>46305</v>
       </c>
-      <c r="D8" t="s">
-        <v>30</v>
+      <c r="D8" s="1">
+        <v>46305</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="G8" t="s">
         <v>83</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="s">
+        <v>84</v>
+      </c>
+      <c r="I8">
         <v>2.95</v>
       </c>
-      <c r="I8" t="s">
-        <v>84</v>
-      </c>
       <c r="J8" t="s">
-        <v>92</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8" t="s">
-        <v>120</v>
+        <v>85</v>
+      </c>
+      <c r="K8" t="s">
+        <v>93</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
       </c>
       <c r="M8" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
       <c r="N8" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+        <v>148</v>
+      </c>
+      <c r="O8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1551,41 +1587,44 @@
       <c r="C9" s="1">
         <v>46305</v>
       </c>
-      <c r="D9" t="s">
-        <v>31</v>
+      <c r="D9" s="1">
+        <v>46305</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="G9" t="s">
         <v>83</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="s">
+        <v>84</v>
+      </c>
+      <c r="I9">
         <v>69.5</v>
       </c>
-      <c r="I9" t="s">
-        <v>84</v>
-      </c>
       <c r="J9" t="s">
-        <v>93</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9" t="s">
-        <v>121</v>
+        <v>85</v>
+      </c>
+      <c r="K9" t="s">
+        <v>94</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>146</v>
+        <v>123</v>
       </c>
       <c r="N9" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+        <v>149</v>
+      </c>
+      <c r="O9" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1595,41 +1634,44 @@
       <c r="C10" s="1">
         <v>46305</v>
       </c>
-      <c r="D10" t="s">
-        <v>32</v>
+      <c r="D10" s="1">
+        <v>46305</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="G10" t="s">
         <v>83</v>
       </c>
-      <c r="H10">
+      <c r="H10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10">
         <v>62.95</v>
       </c>
-      <c r="I10" t="s">
-        <v>84</v>
-      </c>
       <c r="J10" t="s">
-        <v>94</v>
-      </c>
-      <c r="K10">
+        <v>85</v>
+      </c>
+      <c r="K10" t="s">
+        <v>95</v>
+      </c>
+      <c r="L10">
         <v>79</v>
       </c>
-      <c r="L10" t="s">
-        <v>122</v>
-      </c>
       <c r="M10" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="N10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+        <v>147</v>
+      </c>
+      <c r="O10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1639,41 +1681,44 @@
       <c r="C11" s="1">
         <v>46305</v>
       </c>
-      <c r="D11" t="s">
-        <v>33</v>
+      <c r="D11" s="1">
+        <v>46305</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="G11" t="s">
         <v>83</v>
       </c>
-      <c r="H11">
+      <c r="H11" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11">
         <v>134.2</v>
       </c>
-      <c r="I11" t="s">
-        <v>84</v>
-      </c>
       <c r="J11" t="s">
-        <v>95</v>
-      </c>
-      <c r="K11">
+        <v>85</v>
+      </c>
+      <c r="K11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L11">
         <v>1</v>
       </c>
-      <c r="L11" t="s">
-        <v>123</v>
-      </c>
       <c r="M11" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="N11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+        <v>147</v>
+      </c>
+      <c r="O11" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1683,41 +1728,44 @@
       <c r="C12" s="1">
         <v>46305</v>
       </c>
-      <c r="D12" t="s">
-        <v>34</v>
+      <c r="D12" s="1">
+        <v>46305</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="G12" t="s">
         <v>83</v>
       </c>
-      <c r="H12">
+      <c r="H12" t="s">
+        <v>84</v>
+      </c>
+      <c r="I12">
         <v>69.90000000000001</v>
       </c>
-      <c r="I12" t="s">
-        <v>84</v>
-      </c>
       <c r="J12" t="s">
-        <v>96</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12" t="s">
-        <v>124</v>
+        <v>85</v>
+      </c>
+      <c r="K12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="N12" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1727,41 +1775,44 @@
       <c r="C13" s="1">
         <v>46306</v>
       </c>
-      <c r="D13" t="s">
-        <v>35</v>
+      <c r="D13" s="1">
+        <v>46306</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="G13" t="s">
         <v>83</v>
       </c>
-      <c r="H13">
+      <c r="H13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I13">
         <v>29.45</v>
       </c>
-      <c r="I13" t="s">
-        <v>84</v>
-      </c>
       <c r="J13" t="s">
-        <v>97</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13" t="s">
-        <v>125</v>
+        <v>85</v>
+      </c>
+      <c r="K13" t="s">
+        <v>98</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
       </c>
       <c r="M13" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="N13" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O13" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1771,41 +1822,44 @@
       <c r="C14" s="1">
         <v>46306</v>
       </c>
-      <c r="D14" t="s">
-        <v>36</v>
+      <c r="D14" s="1">
+        <v>46306</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="G14" t="s">
         <v>83</v>
       </c>
-      <c r="H14">
+      <c r="H14" t="s">
+        <v>84</v>
+      </c>
+      <c r="I14">
         <v>29.95</v>
       </c>
-      <c r="I14" t="s">
-        <v>84</v>
-      </c>
       <c r="J14" t="s">
-        <v>98</v>
-      </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14" t="s">
-        <v>126</v>
+        <v>85</v>
+      </c>
+      <c r="K14" t="s">
+        <v>99</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="N14" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+        <v>150</v>
+      </c>
+      <c r="O14" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1815,41 +1869,44 @@
       <c r="C15" s="1">
         <v>46306</v>
       </c>
-      <c r="D15" t="s">
-        <v>37</v>
+      <c r="D15" s="1">
+        <v>46306</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
         <v>83</v>
       </c>
-      <c r="H15">
+      <c r="H15" t="s">
+        <v>84</v>
+      </c>
+      <c r="I15">
         <v>105.4</v>
       </c>
-      <c r="I15" t="s">
-        <v>84</v>
-      </c>
       <c r="J15" t="s">
-        <v>99</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15" t="s">
-        <v>127</v>
+        <v>85</v>
+      </c>
+      <c r="K15" t="s">
+        <v>100</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
       </c>
       <c r="M15" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="N15" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -1859,41 +1916,44 @@
       <c r="C16" s="1">
         <v>46306</v>
       </c>
-      <c r="D16" t="s">
-        <v>38</v>
+      <c r="D16" s="1">
+        <v>46306</v>
       </c>
       <c r="E16" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G16" t="s">
         <v>83</v>
       </c>
-      <c r="H16">
+      <c r="H16" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16">
         <v>105.5</v>
       </c>
-      <c r="I16" t="s">
-        <v>84</v>
-      </c>
       <c r="J16" t="s">
-        <v>100</v>
-      </c>
-      <c r="K16">
+        <v>85</v>
+      </c>
+      <c r="K16" t="s">
+        <v>101</v>
+      </c>
+      <c r="L16">
         <v>71</v>
       </c>
-      <c r="L16" t="s">
-        <v>128</v>
-      </c>
       <c r="M16" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="N16" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14">
+        <v>150</v>
+      </c>
+      <c r="O16" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -1903,41 +1963,44 @@
       <c r="C17" s="1">
         <v>46306</v>
       </c>
-      <c r="D17" t="s">
-        <v>39</v>
+      <c r="D17" s="1">
+        <v>46306</v>
       </c>
       <c r="E17" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="G17" t="s">
         <v>83</v>
       </c>
-      <c r="H17">
+      <c r="H17" t="s">
+        <v>84</v>
+      </c>
+      <c r="I17">
         <v>77.5</v>
       </c>
-      <c r="I17" t="s">
-        <v>84</v>
-      </c>
       <c r="J17" t="s">
-        <v>101</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17" t="s">
-        <v>129</v>
+        <v>85</v>
+      </c>
+      <c r="K17" t="s">
+        <v>102</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
       </c>
       <c r="M17" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="N17" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O17" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1947,41 +2010,44 @@
       <c r="C18" s="1">
         <v>46306</v>
       </c>
-      <c r="D18" t="s">
-        <v>40</v>
+      <c r="D18" s="1">
+        <v>46306</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="F18" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="G18" t="s">
         <v>83</v>
       </c>
-      <c r="H18">
+      <c r="H18" t="s">
+        <v>84</v>
+      </c>
+      <c r="I18">
         <v>54.45</v>
       </c>
-      <c r="I18" t="s">
-        <v>84</v>
-      </c>
       <c r="J18" t="s">
-        <v>102</v>
-      </c>
-      <c r="K18">
+        <v>85</v>
+      </c>
+      <c r="K18" t="s">
+        <v>103</v>
+      </c>
+      <c r="L18">
         <v>28</v>
       </c>
-      <c r="L18" t="s">
-        <v>130</v>
-      </c>
       <c r="M18" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="N18" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -1991,41 +2057,44 @@
       <c r="C19" s="1">
         <v>46306</v>
       </c>
-      <c r="D19" t="s">
-        <v>41</v>
+      <c r="D19" s="1">
+        <v>46306</v>
       </c>
       <c r="E19" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="F19" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="G19" t="s">
         <v>83</v>
       </c>
-      <c r="H19">
+      <c r="H19" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19">
         <v>59.5</v>
       </c>
-      <c r="I19" t="s">
-        <v>84</v>
-      </c>
       <c r="J19" t="s">
-        <v>103</v>
-      </c>
-      <c r="K19">
+        <v>85</v>
+      </c>
+      <c r="K19" t="s">
+        <v>104</v>
+      </c>
+      <c r="L19">
         <v>76</v>
       </c>
-      <c r="L19" t="s">
-        <v>131</v>
-      </c>
       <c r="M19" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="N19" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -2035,41 +2104,44 @@
       <c r="C20" s="1">
         <v>46306</v>
       </c>
-      <c r="D20" t="s">
-        <v>42</v>
+      <c r="D20" s="1">
+        <v>46306</v>
       </c>
       <c r="E20" t="s">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="F20" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="G20" t="s">
         <v>83</v>
       </c>
-      <c r="H20">
+      <c r="H20" t="s">
+        <v>84</v>
+      </c>
+      <c r="I20">
         <v>7.7</v>
       </c>
-      <c r="I20" t="s">
-        <v>84</v>
-      </c>
       <c r="J20" t="s">
-        <v>104</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20" t="s">
-        <v>132</v>
+        <v>85</v>
+      </c>
+      <c r="K20" t="s">
+        <v>105</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
       </c>
       <c r="M20" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="N20" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14">
+        <v>148</v>
+      </c>
+      <c r="O20" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -2079,41 +2151,44 @@
       <c r="C21" s="1">
         <v>46307</v>
       </c>
-      <c r="D21" t="s">
-        <v>43</v>
+      <c r="D21" s="1">
+        <v>46307</v>
       </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="F21" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="G21" t="s">
         <v>83</v>
       </c>
-      <c r="H21">
+      <c r="H21" t="s">
+        <v>84</v>
+      </c>
+      <c r="I21">
         <v>59.9</v>
       </c>
-      <c r="I21" t="s">
-        <v>84</v>
-      </c>
       <c r="J21" t="s">
-        <v>105</v>
-      </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21" t="s">
-        <v>133</v>
+        <v>85</v>
+      </c>
+      <c r="K21" t="s">
+        <v>106</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
       </c>
       <c r="M21" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="N21" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O21" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -2123,41 +2198,44 @@
       <c r="C22" s="1">
         <v>46307</v>
       </c>
-      <c r="D22" t="s">
-        <v>44</v>
+      <c r="D22" s="1">
+        <v>46307</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="F22" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="G22" t="s">
         <v>83</v>
       </c>
-      <c r="H22">
+      <c r="H22" t="s">
+        <v>84</v>
+      </c>
+      <c r="I22">
         <v>41.95</v>
       </c>
-      <c r="I22" t="s">
-        <v>84</v>
-      </c>
       <c r="J22" t="s">
-        <v>106</v>
-      </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-      <c r="L22" t="s">
-        <v>134</v>
+        <v>85</v>
+      </c>
+      <c r="K22" t="s">
+        <v>107</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
       </c>
       <c r="M22" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="N22" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O22" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -2167,41 +2245,44 @@
       <c r="C23" s="1">
         <v>46307</v>
       </c>
-      <c r="D23" t="s">
-        <v>45</v>
+      <c r="D23" s="1">
+        <v>46307</v>
       </c>
       <c r="E23" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="F23" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G23" t="s">
         <v>83</v>
       </c>
-      <c r="H23">
+      <c r="H23" t="s">
+        <v>84</v>
+      </c>
+      <c r="I23">
         <v>95.90000000000001</v>
       </c>
-      <c r="I23" t="s">
-        <v>84</v>
-      </c>
       <c r="J23" t="s">
-        <v>107</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23" t="s">
-        <v>135</v>
+        <v>85</v>
+      </c>
+      <c r="K23" t="s">
+        <v>108</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
       </c>
       <c r="M23" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="N23" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O23" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -2211,41 +2292,44 @@
       <c r="C24" s="1">
         <v>46307</v>
       </c>
-      <c r="D24" t="s">
-        <v>46</v>
+      <c r="D24" s="1">
+        <v>46307</v>
       </c>
       <c r="E24" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G24" t="s">
         <v>83</v>
       </c>
-      <c r="H24">
+      <c r="H24" t="s">
+        <v>84</v>
+      </c>
+      <c r="I24">
         <v>48.25</v>
       </c>
-      <c r="I24" t="s">
-        <v>84</v>
-      </c>
       <c r="J24" t="s">
-        <v>108</v>
-      </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
-      <c r="L24" t="s">
-        <v>136</v>
+        <v>85</v>
+      </c>
+      <c r="K24" t="s">
+        <v>109</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
       </c>
       <c r="M24" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="N24" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14">
+        <v>149</v>
+      </c>
+      <c r="O24" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -2255,41 +2339,44 @@
       <c r="C25" s="1">
         <v>46307</v>
       </c>
-      <c r="D25" t="s">
-        <v>47</v>
+      <c r="D25" s="1">
+        <v>46307</v>
       </c>
       <c r="E25" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="G25" t="s">
         <v>83</v>
       </c>
-      <c r="H25">
+      <c r="H25" t="s">
+        <v>84</v>
+      </c>
+      <c r="I25">
         <v>74.45</v>
       </c>
-      <c r="I25" t="s">
-        <v>84</v>
-      </c>
       <c r="J25" t="s">
-        <v>109</v>
-      </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25" t="s">
-        <v>137</v>
+        <v>85</v>
+      </c>
+      <c r="K25" t="s">
+        <v>110</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
       </c>
       <c r="M25" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N25" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14">
+        <v>145</v>
+      </c>
+      <c r="O25" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -2299,41 +2386,44 @@
       <c r="C26" s="1">
         <v>46307</v>
       </c>
-      <c r="D26" t="s">
-        <v>48</v>
+      <c r="D26" s="1">
+        <v>46307</v>
       </c>
       <c r="E26" t="s">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="F26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G26" t="s">
         <v>83</v>
       </c>
-      <c r="H26">
+      <c r="H26" t="s">
+        <v>84</v>
+      </c>
+      <c r="I26">
         <v>67.15000000000001</v>
       </c>
-      <c r="I26" t="s">
-        <v>84</v>
-      </c>
       <c r="J26" t="s">
-        <v>110</v>
-      </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-      <c r="L26" t="s">
-        <v>138</v>
+        <v>85</v>
+      </c>
+      <c r="K26" t="s">
+        <v>111</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
       </c>
       <c r="M26" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="N26" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14">
+        <v>149</v>
+      </c>
+      <c r="O26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -2343,26 +2433,44 @@
       <c r="C27" s="1">
         <v>46307</v>
       </c>
-      <c r="D27" t="s">
-        <v>49</v>
+      <c r="D27" s="1">
+        <v>46307</v>
       </c>
       <c r="E27" t="s">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="F27" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G27" t="s">
         <v>83</v>
       </c>
-      <c r="H27">
+      <c r="H27" t="s">
+        <v>84</v>
+      </c>
+      <c r="I27">
         <v>59.5</v>
       </c>
-      <c r="I27" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14">
+      <c r="J27" t="s">
+        <v>86</v>
+      </c>
+      <c r="K27" t="s">
+        <v>112</v>
+      </c>
+      <c r="L27">
+        <v>1510</v>
+      </c>
+      <c r="M27" t="s">
+        <v>141</v>
+      </c>
+      <c r="N27" t="s">
+        <v>150</v>
+      </c>
+      <c r="O27" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -2372,41 +2480,44 @@
       <c r="C28" s="1">
         <v>46308</v>
       </c>
-      <c r="D28" t="s">
-        <v>50</v>
+      <c r="D28" s="1">
+        <v>46308</v>
       </c>
       <c r="E28" t="s">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="F28" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G28" t="s">
         <v>83</v>
       </c>
-      <c r="H28">
+      <c r="H28" t="s">
+        <v>84</v>
+      </c>
+      <c r="I28">
         <v>59.9</v>
       </c>
-      <c r="I28" t="s">
-        <v>84</v>
-      </c>
       <c r="J28" t="s">
-        <v>111</v>
-      </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
-      <c r="L28" t="s">
-        <v>139</v>
+        <v>85</v>
+      </c>
+      <c r="K28" t="s">
+        <v>113</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
       </c>
       <c r="M28" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N28" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O28" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -2416,41 +2527,44 @@
       <c r="C29" s="1">
         <v>46309</v>
       </c>
-      <c r="D29" t="s">
-        <v>51</v>
+      <c r="D29" s="1">
+        <v>46309</v>
       </c>
       <c r="E29" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="F29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G29" t="s">
         <v>83</v>
       </c>
-      <c r="H29">
+      <c r="H29" t="s">
+        <v>84</v>
+      </c>
+      <c r="I29">
         <v>105.6</v>
       </c>
-      <c r="I29" t="s">
-        <v>84</v>
-      </c>
       <c r="J29" t="s">
-        <v>112</v>
-      </c>
-      <c r="K29">
+        <v>85</v>
+      </c>
+      <c r="K29" t="s">
+        <v>114</v>
+      </c>
+      <c r="L29">
         <v>1</v>
-      </c>
-      <c r="L29" t="s">
-        <v>140</v>
       </c>
       <c r="M29" t="s">
         <v>143</v>
       </c>
       <c r="N29" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14">
+        <v>146</v>
+      </c>
+      <c r="O29" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -2460,11 +2574,11 @@
       <c r="C30" s="1">
         <v>46309</v>
       </c>
-      <c r="D30" t="s">
-        <v>52</v>
+      <c r="D30" s="1">
+        <v>46309</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="F30" t="s">
         <v>82</v>
@@ -2472,26 +2586,29 @@
       <c r="G30" t="s">
         <v>83</v>
       </c>
-      <c r="H30">
+      <c r="H30" t="s">
+        <v>84</v>
+      </c>
+      <c r="I30">
         <v>44.75</v>
       </c>
-      <c r="I30" t="s">
-        <v>84</v>
-      </c>
       <c r="J30" t="s">
-        <v>113</v>
-      </c>
-      <c r="K30">
-        <v>0</v>
-      </c>
-      <c r="L30" t="s">
-        <v>141</v>
+        <v>85</v>
+      </c>
+      <c r="K30" t="s">
+        <v>115</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
       </c>
       <c r="M30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N30" t="s">
-        <v>174</v>
+        <v>148</v>
+      </c>
+      <c r="O30" t="s">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2501,10 +2618,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2547,8 +2664,11 @@
       <c r="N1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2558,23 +2678,41 @@
       <c r="C2" s="1">
         <v>46307</v>
       </c>
-      <c r="D2" t="s">
-        <v>49</v>
+      <c r="D2" s="1">
+        <v>46307</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G2" t="s">
         <v>83</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2">
         <v>59.5</v>
       </c>
-      <c r="I2" t="s">
-        <v>85</v>
+      <c r="J2" t="s">
+        <v>86</v>
+      </c>
+      <c r="K2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2">
+        <v>1510</v>
+      </c>
+      <c r="M2" t="s">
+        <v>141</v>
+      </c>
+      <c r="N2" t="s">
+        <v>150</v>
+      </c>
+      <c r="O2" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -2598,25 +2736,25 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="I1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="J1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2640,25 +2778,25 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="I1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="J1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>